<commit_message>
Schlusspruefung: Korrekturen gegen die Quellen
Automatisch nach dem Erstellen geprueft. Einzelheiten im Kommentar des Pull Requests.
</commit_message>
<xml_diff>
--- a/vorlagen/wartungskalender-instandhaltung-wohngebaeude/wartungskalender-instandhaltung-wohngebaeude.xlsx
+++ b/vorlagen/wartungskalender-instandhaltung-wohngebaeude/wartungskalender-instandhaltung-wohngebaeude.xlsx
@@ -822,7 +822,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>DIN 18531, Wartung</t>
+          <t>Flachdachrichtlinie, Abschnitt Wartung</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>DIN 18531, Wartung</t>
+          <t>Flachdachrichtlinie, Abschnitt Wartung</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>einmal jährlich und vor jeder Nutzung</t>
+          <t>vor jeder Nutzung sichten, Prüfintervall nach Herstellerangabe</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -1617,12 +1617,12 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>zweimal jährlich, bei Trockenheit häufiger</t>
+          <t>Intervall nach DIN 1986-3 festlegen, bei Trockenheit häufiger</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>DIN 1986-3, Wartungshinweis</t>
+          <t>DIN 1986-3, Regeln für Betrieb und Wartung</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -1657,12 +1657,12 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>zweimal jährlich, nach dem Laubfall</t>
+          <t>Intervall nach DIN 1986-3 festlegen, zusätzlich nach dem Laubfall</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>DIN 1986-3</t>
+          <t>DIN 1986-3, Regeln für Betrieb und Wartung</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>bei jeder Untersuchung, Meldung innerhalb von zwei Wochen</t>
+          <t>bei jeder Untersuchung, Meldung bei Überschreitung des technischen Maßnahmenwerts</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -2257,12 +2257,12 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Intervall nach VDI 6022 Blatt 1 und Anlagenart festlegen</t>
+          <t>Intervall nach Anlagenart und Herstellerangabe festlegen</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>VDI 6022 Blatt 1</t>
+          <t>Herstellerangabe, Hygieneinspektion der Lüftungsanlage</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>DIN 14406-4, Instandhaltung tragbarer Feuerlöscher</t>
+          <t>Instandhaltung tragbarer Feuerlöscher, Prüfnachweis am Gerät</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
@@ -3582,7 +3582,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>DIN 31051, Dokumentation der Instandhaltung</t>
+          <t>Nachweisführung in der Gebäudeakte</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>Verkehrssicherungspflicht bei Übertragung und Überwachung</t>
+          <t>Betreiberorganisation</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -3987,7 +3987,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>• Legen Sie zu jeder ausgeführten Leistung den Bericht, die Bescheinigung oder das Protokoll in der Gebäudeakte ab. Eine Leistung ohne Nachweis gilt im Streitfall als nicht erbracht.</t>
+          <t>• Legen Sie zu jeder ausgeführten Leistung den Bericht, die Bescheinigung oder das Protokoll in der Gebäudeakte ab. Eine Leistung ohne Nachweis lässt sich später nicht belegen.</t>
         </is>
       </c>
     </row>
@@ -4022,7 +4022,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>• Die Übertragung von Aufgaben an Hausmeister oder Fachbetriebe entlastet nur, wenn sie schriftlich geregelt und die Ausführung kontrolliert wird.</t>
+          <t>• Regeln Sie die Übertragung von Aufgaben an Hausmeister oder Fachbetriebe schriftlich und kontrollieren Sie die Ausführung.</t>
         </is>
       </c>
     </row>
@@ -4036,7 +4036,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Grundlagen: Wartung von Dachabdichtungen zweimal jährlich und Schutz der Abläufe durch Laubfangkörbe (Flachdachrichtlinie 2017, Abschnitt 5.4 und 4.1, zitiert bei Schulz: Architektur der Bauschäden, 4. Aufl. 2020, S. 152) · Inspektion und Wartung der Abdichtung von Dächern, Balkonen und Terrassen mindestens einmal jährlich durch ein Fachunternehmen, Dokumentation, Reinigung von Gullys, Dachrinnen und Fallrohren (Weber/Hafkesbrink: Bauwerksabdichtung in der Altbausanierung, 7. Aufl. 2026, S. 453 f., zu DIN 18531-4) · Wartung von Balkonen, Loggien und Laubengängen mindestens einmal jährlich im Zusammenhang mit einer Inspektion (DIN 18531-5, Abschnitt 11.3, zitiert bei Schulz: Architektur der Bauschäden, 4. Aufl. 2020, S. 151) · Kontrolle und Prüfung von Rückstauverschlüssen zweimal im Jahr, bei Typ 3 durch fachkundiges Personal (DIN EN 13564-1, Anhang B, zitiert bei Schulz: Architektur der Bauschäden, 4. Aufl. 2020, S. 192) · Zeitintervalle der regelmäßigen Überprüfung der Standsicherheit, Schadensfolgeklassen und Checkliste der Schadensindizien (VDI 6200, wiedergegeben in Wendehorst Bautechnische Zahlentafeln, 37. Aufl. 2021, S. 1085 bis 1091) · Pflicht des Betreibers zur regelmäßigen Wartung und Instandhaltung, Fachkunde, Empfehlung der jährlichen Heizungswartung vor der Heizperiode sowie Betriebsprüfung von Wärmepumpen (GEG § 58, § 59, § 60 und § 60a, wiedergegeben bei Schmidt: Das novellierte Gebäudeenergiegesetz, 2025, S. 236 bis 238) · Untersuchungspflicht auf Legionellen, betroffene Anlagen, Intervalle und Verantwortung von Vermieter und Hausverwaltung (Landesamt für Gesundheit und Soziales Berlin, Trinkwasserhygiene, Legionellen in Hausinstallationen) · Prüffrist der Hauptprüfung von Aufzugsanlagen von höchstens zwei Jahren und Zweiwege-Kommunikationssystem (Deutsche Gesetzliche Unfallversicherung, FAQ zu Aufzügen, zu Anhang 2 Abschnitt 2 der Betriebssicherheitsverordnung) · Inspektion von Rauchwarnmeldern alle zwölf Monate, abweichende Fristen bei Ferninspektion (DIN 14676-1 in der Ausgabe 2025-05, DIN Media; Inspektionszeiträume nach BundesBauBlatt) · Inspektion, Wartung und Betrieb von Spielplatzgeräten (DIN EN 1176-7 in der Ausgabe 2020-06, DIN Media; Kontrollintervalle nach Hinweisen der Deutschen Gesetzlichen Unfallversicherung) · Regelkontrollen zur Überprüfung der Verkehrssicherheit von Bäumen (FLL-Baumkontrollrichtlinien, Ausgabe 2020, Forschungsgesellschaft Landschaftsentwicklung Landschaftsbau) · Begriffe Instandhaltung, Wartung, Inspektion und Instandsetzung (DIN 31051 in der Ausgabe 2019-06, DIN Media; zitiert bei Schulz 2020, S. 151, und Schmidt/Windhausen: Lohmeyer Praktische Bauphysik, 10. Aufl. 2024, S. 408) · Sicherheitstechnische Anforderungen an Arbeitsplätze und Verkehrswege für die Instandhaltung baulicher Anlagen (DIN 4426 in der Ausgabe 2017-01, DIN Media) · Regeln für Betrieb und Wartung von Entwässerungsanlagen (DIN 1986-3 in der Ausgabe 2024-05, DIN Media) · Instandhaltungsplanung mit Einordnung in kurz-, mittel- und langfristige Maßnahmen (Schulz: Architektur der Bauschäden, 4. Aufl. 2020, S. 581 bis 584)</t>
+          <t>Grundlagen: Wartung von Dachabdichtungen zweimal jährlich und Schutz der Abläufe durch Laubfangkörbe (Flachdachrichtlinie 2017, Abschnitt 5.4 und 4.1, zitiert bei Schulz: Architektur der Bauschäden, 4. Aufl. 2020, S. 152) · Inspektion und Wartung der Abdichtung von Dächern, Balkonen und Terrassen mindestens einmal jährlich durch ein Fachunternehmen, Dokumentation, Reinigung von Gullys, Dachrinnen und Fallrohren (Weber/Hafkesbrink: Bauwerksabdichtung in der Altbausanierung, 7. Aufl. 2026, S. 453 f., zu DIN 18531-4) · Wartung von Balkonen, Loggien und Laubengängen mindestens einmal jährlich im Zusammenhang mit einer Inspektion (DIN 18531-5, Abschnitt 11.3, zitiert bei Schulz: Architektur der Bauschäden, 4. Aufl. 2020, S. 151) · Kontrolle und Prüfung von Rückstauverschlüssen zweimal im Jahr, bei Typ 3 durch fachkundiges Personal (DIN EN 13564-1, Anhang B, zitiert bei Schulz: Architektur der Bauschäden, 4. Aufl. 2020, S. 192) · Zeitintervalle der regelmäßigen Überprüfung der Standsicherheit, Schadensfolgeklassen und Checkliste der Schadensindizien (VDI 6200, wiedergegeben in Wendehorst Bautechnische Zahlentafeln, 37. Aufl. 2021, S. 1085 bis 1091) · Pflicht des Betreibers zur regelmäßigen Wartung und Instandhaltung, Fachkunde, Empfehlung der jährlichen Heizungswartung vor der Heizperiode sowie Betriebsprüfung von Wärmepumpen (GEG § 58, § 59, § 60 und § 60a, wiedergegeben bei Schmidt: Das novellierte Gebäudeenergiegesetz, 2025, S. 236 bis 238) · Untersuchungspflicht auf Legionellen, betroffene Anlagen, Intervalle und Verantwortung von Vermieter und Hausverwaltung (Landesamt für Gesundheit und Soziales Berlin, Trinkwasserhygiene, Legionellen in Hausinstallationen) · Prüffrist der Hauptprüfung von Aufzugsanlagen von höchstens zwei Jahren und Zweiwege-Kommunikationssystem (Deutsche Gesetzliche Unfallversicherung, FAQ zu Aufzügen, zu Anhang 2 Abschnitt 2 der Betriebssicherheitsverordnung) · Inspektion von Rauchwarnmeldern alle zwölf Monate, abweichende Fristen bei Ferninspektion (DIN 14676-1 in der Ausgabe 2025-05, DIN Media; Inspektionszeiträume nach BundesBauBlatt) · Inspektion, Wartung und Betrieb von Spielplatzgeräten (DIN EN 1176-7 in der Ausgabe 2020-06, DIN Media; Kontrollintervalle nach Hinweisen der Deutschen Gesetzlichen Unfallversicherung) · Regelkontrollen zur Überprüfung der Verkehrssicherheit von Bäumen (FLL-Baumkontrollrichtlinien, Ausgabe 2020, Forschungsgesellschaft Landschaftsentwicklung Landschaftsbau) · Begriffe Instandhaltung, Wartung, Inspektion und Instandsetzung (DIN 31051 in der Ausgabe 2019-06, DIN Media; zitiert bei Schulz 2020, S. 151, und Schmidt/Windhausen: Lohmeyer Praktische Bauphysik, 10. Aufl. 2024, S. 408) · Sicherheitstechnische Anforderungen an Arbeitsplätze und Verkehrswege für die Instandhaltung baulicher Anlagen (DIN 4426, zitiert bei Schulz: Architektur der Bauschäden, 4. Aufl. 2020, S. 152) · Regeln für Betrieb und Wartung von Entwässerungsanlagen (DIN 1986-3 in der Ausgabe 2024-05, DIN Media) · Instandhaltungsplanung mit Einordnung in kurz-, mittel- und langfristige Maßnahmen (Schulz: Architektur der Bauschäden, 4. Aufl. 2020, S. 581 bis 584)</t>
         </is>
       </c>
     </row>

</xml_diff>